<commit_message>
mejora en la documentación
</commit_message>
<xml_diff>
--- a/CheckList Examen/Checklist Examen.xlsx
+++ b/CheckList Examen/Checklist Examen.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Home\Desktop\4. Spring Cloud\0. Repositorio - Consolidado\EVALUACION_FINAL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Home\Desktop\4. Spring Cloud\0. [MIRKO] - EVALUACION_FINAL\Documentacion\CheckList Examen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5F32839-309F-441A-863C-1ED67BAA552D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D915BA81-AAF2-4EDB-8A58-2C7F204119FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{47D30B52-2BD7-4906-9AF6-B7407B7A6AF9}"/>
+    <workbookView xWindow="6324" yWindow="540" windowWidth="23040" windowHeight="11664" xr2:uid="{47D30B52-2BD7-4906-9AF6-B7407B7A6AF9}"/>
   </bookViews>
   <sheets>
     <sheet name="Requisitos Generales" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="24">
   <si>
     <t>Caso de negocio</t>
   </si>
@@ -80,6 +80,15 @@
     <t>Mensajería (Kafka)</t>
   </si>
   <si>
+    <t>Seguridad:</t>
+  </si>
+  <si>
+    <t>Validación de token</t>
+  </si>
+  <si>
+    <t>PreAuthorize</t>
+  </si>
+  <si>
     <t>Documentación y Observabilidad:</t>
   </si>
   <si>
@@ -99,6 +108,9 @@
   </si>
   <si>
     <t>Microservicios levantados desde IDE</t>
+  </si>
+  <si>
+    <t>Servicio de autenticación generador de token JWT</t>
   </si>
 </sst>
 </file>
@@ -515,18 +527,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9C2F772-FA25-43B8-A864-CA9DE157B618}">
-  <dimension ref="B3:E18"/>
+  <dimension ref="B3:E22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="50.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="9.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" s="2"/>
       <c r="C3" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>2</v>
@@ -664,7 +676,7 @@
     <row r="13" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B13" s="2"/>
       <c r="C13" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>2</v>
@@ -678,7 +690,7 @@
         <v>10</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>7</v>
@@ -692,7 +704,7 @@
         <v>11</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>8</v>
@@ -704,7 +716,7 @@
     <row r="16" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>2</v>
@@ -718,7 +730,7 @@
         <v>12</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>7</v>
@@ -732,12 +744,66 @@
         <v>13</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>7</v>
       </c>
       <c r="E18" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B19" s="2"/>
+      <c r="C19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B20" s="4">
+        <v>14</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B21" s="4">
+        <v>15</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B22" s="4">
+        <v>16</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>